<commit_message>
add excel config file
</commit_message>
<xml_diff>
--- a/Immagini/prodotti season 72.20.05.2026.xlsx
+++ b/Immagini/prodotti season 72.20.05.2026.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="6">
   <si>
     <t>Option</t>
   </si>
@@ -44,7 +44,7 @@
     <t>Needed?</t>
   </si>
   <si>
-    <t>N</t>
+    <t>Y</t>
   </si>
 </sst>
 </file>
@@ -5818,9 +5818,8 @@
       <c r="C397">
         <v>3083</v>
       </c>
-      <c r="E397" s="4" t="str">
-        <f t="shared" ref="E387:E450" si="0">+IF(B397&lt;&gt;"","Y","")</f>
-        <v>Y</v>
+      <c r="E397" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="398" spans="2:5">
@@ -5830,9 +5829,8 @@
       <c r="C398">
         <v>3270</v>
       </c>
-      <c r="E398" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E398" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="399" spans="2:5">
@@ -5842,9 +5840,8 @@
       <c r="C399">
         <v>7005</v>
       </c>
-      <c r="E399" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E399" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="400" spans="2:5">
@@ -5854,9 +5851,8 @@
       <c r="C400">
         <v>2416</v>
       </c>
-      <c r="E400" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E400" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="401" spans="2:5">
@@ -5866,9 +5862,8 @@
       <c r="C401">
         <v>3083</v>
       </c>
-      <c r="E401" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E401" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="402" spans="2:5">
@@ -5878,9 +5873,8 @@
       <c r="C402">
         <v>3270</v>
       </c>
-      <c r="E402" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E402" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="403" spans="2:5">
@@ -5890,9 +5884,8 @@
       <c r="C403">
         <v>7005</v>
       </c>
-      <c r="E403" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E403" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="404" spans="2:5">
@@ -5902,9 +5895,8 @@
       <c r="C404">
         <v>2416</v>
       </c>
-      <c r="E404" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E404" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="405" spans="2:5">
@@ -5914,9 +5906,8 @@
       <c r="C405">
         <v>3083</v>
       </c>
-      <c r="E405" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E405" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="406" spans="2:5">
@@ -5926,9 +5917,8 @@
       <c r="C406">
         <v>3270</v>
       </c>
-      <c r="E406" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E406" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="407" spans="2:5">
@@ -5938,9 +5928,8 @@
       <c r="C407">
         <v>7005</v>
       </c>
-      <c r="E407" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E407" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="408" spans="2:5">
@@ -5950,9 +5939,8 @@
       <c r="C408">
         <v>3083</v>
       </c>
-      <c r="E408" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E408" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="409" spans="2:5">
@@ -5962,9 +5950,8 @@
       <c r="C409">
         <v>3270</v>
       </c>
-      <c r="E409" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E409" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="410" spans="2:5">
@@ -5974,9 +5961,8 @@
       <c r="C410">
         <v>7005</v>
       </c>
-      <c r="E410" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E410" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="411" spans="2:5">
@@ -5986,9 +5972,8 @@
       <c r="C411">
         <v>3083</v>
       </c>
-      <c r="E411" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E411" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="412" spans="2:5">
@@ -5998,9 +5983,8 @@
       <c r="C412">
         <v>3270</v>
       </c>
-      <c r="E412" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E412" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="413" spans="2:5">
@@ -6010,9 +5994,8 @@
       <c r="C413">
         <v>7005</v>
       </c>
-      <c r="E413" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E413" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="414" spans="2:5">
@@ -6022,9 +6005,8 @@
       <c r="C414">
         <v>3083</v>
       </c>
-      <c r="E414" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E414" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="415" spans="2:5">
@@ -6034,9 +6016,8 @@
       <c r="C415">
         <v>7005</v>
       </c>
-      <c r="E415" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E415" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="416" spans="2:5">
@@ -6046,9 +6027,8 @@
       <c r="C416">
         <v>7539</v>
       </c>
-      <c r="E416" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E416" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="417" spans="2:5">
@@ -6058,9 +6038,8 @@
       <c r="C417">
         <v>3083</v>
       </c>
-      <c r="E417" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E417" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="418" spans="2:5">
@@ -6070,9 +6049,8 @@
       <c r="C418">
         <v>7005</v>
       </c>
-      <c r="E418" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E418" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="419" spans="2:5">
@@ -6082,9 +6060,8 @@
       <c r="C419">
         <v>7539</v>
       </c>
-      <c r="E419" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E419" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="420" spans="2:5">
@@ -6094,9 +6071,8 @@
       <c r="C420">
         <v>7005</v>
       </c>
-      <c r="E420" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E420" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="421" spans="2:5">
@@ -6106,9 +6082,8 @@
       <c r="C421">
         <v>7539</v>
       </c>
-      <c r="E421" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E421" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="422" spans="2:5">
@@ -6118,9 +6093,8 @@
       <c r="C422">
         <v>8240</v>
       </c>
-      <c r="E422" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E422" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="423" spans="2:5">
@@ -6130,9 +6104,8 @@
       <c r="C423">
         <v>8249</v>
       </c>
-      <c r="E423" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E423" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="424" spans="2:5">
@@ -6142,9 +6115,8 @@
       <c r="C424">
         <v>8240</v>
       </c>
-      <c r="E424" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E424" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="425" spans="2:5">
@@ -6154,9 +6126,8 @@
       <c r="C425">
         <v>8249</v>
       </c>
-      <c r="E425" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E425" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="426" spans="2:5">
@@ -6166,9 +6137,8 @@
       <c r="C426">
         <v>2416</v>
       </c>
-      <c r="E426" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E426" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="427" spans="2:5">
@@ -6178,9 +6148,8 @@
       <c r="C427">
         <v>3083</v>
       </c>
-      <c r="E427" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Y</v>
+      <c r="E427" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="428" spans="2:5">
@@ -6191,7 +6160,7 @@
         <v>7005</v>
       </c>
       <c r="E428" s="4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E397:E450" si="0">+IF(B428&lt;&gt;"","Y","")</f>
         <v>Y</v>
       </c>
     </row>

</xml_diff>